<commit_message>
tirando envio de email
</commit_message>
<xml_diff>
--- a/data/cenarios_demo.xlsx
+++ b/data/cenarios_demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasserranorocco/Documents/DemoApiAutomation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D03A460-A52C-DE4C-A5B0-CF398161AC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{551C6058-0EBE-6341-9199-75EE5CEDC1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7100" yWindow="3120" windowWidth="27840" windowHeight="16740" xr2:uid="{415C9C36-2B63-9848-BD0B-B660EAFFA638}"/>
+    <workbookView xWindow="1900" yWindow="740" windowWidth="27500" windowHeight="10800" xr2:uid="{415C9C36-2B63-9848-BD0B-B660EAFFA638}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>

</xml_diff>